<commit_message>
feat(F002): validated environment schema
src/lib/env.ts: a single Zod schema for every env var read anywhere in this
codebase, replacing scattered process.env.X reads in connection.ts,
auth-pool.ts, auth.ts, and ai-grading.ts. Required vars (DATABASE_URL,
BETTER_AUTH_SECRET, BETTER_AUTH_URL) fail loudly at process boot with the
exact missing key named; optional vars (GOOGLE_CLIENT_ID/SECRET,
ANTHROPIC_API_KEY) match their existing graceful-degradation paths.

Verified live: removing BETTER_AUTH_SECRET from .env throws immediately
with a clear message naming that key, instead of failing confusingly deep
inside a request handler the first time something tries to use it; the app
boots and actually serves a request normally with a correct .env.

.env.example now documents ANTHROPIC_API_KEY, which it was missing.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ExamPrep_AI_Module_Development_Plan.xlsx
+++ b/docs/ExamPrep_AI_Module_Development_Plan.xlsx
@@ -11098,10 +11098,14 @@
       </c>
       <c r="J5" s="72" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K5" s="67" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K5" s="67" t="inlineStr">
+        <is>
+          <t>src/lib/env.ts: a single Zod schema for every env var actually read anywhere in the codebase (DATABASE_URL, BETTER_AUTH_SECRET/URL required; GOOGLE_CLIENT_ID/SECRET and ANTHROPIC_API_KEY optional, matching their documented graceful-degradation paths). Replaced every scattered process.env.X read (connection.ts, auth-pool.ts, auth.ts, ai-grading.ts) with this validated object. Verified live: booting with BETTER_AUTH_SECRET removed throws immediately with the exact missing key named, not a confusing failure deep in a request; booting normally still works, confirmed via a live dev-server request. .env.example already existed and now documents ANTHROPIC_API_KEY too. "Secrets stored in Vercel, never in git" -- .env is already gitignored (verified back in F001) and no secret has been committed at any point this project.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="23.25" customHeight="1" s="59">
       <c r="A6" s="67" t="inlineStr">

</xml_diff>

<commit_message>
feat(F096): close the last cross-household gap -- regenerate-slot
Adds a second fixture question of identical shape (same concept/
bloom/marks/type) so POST /api/papers/:id/regenerate-slot has an
eligible swap target, then asserts a second household gets 404 and
the owning household gets a real 200 with the slot actually swapped
to the alternate question.

This was the one route F096's own note flagged as unswept. With it
covered, the automated suite now exercises every household-scoped
route in the app (17 tests total) -- F096 moves to Done. Global/
admin content routes (questions, syllabus, blueprints CRUD) stay out
of scope since they aren't household-owned data.

Verified live against the real Supabase dev DB: full suite green
(62 tests), zero leftover fixture rows after cleanup.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ExamPrep_AI_Module_Development_Plan.xlsx
+++ b/docs/ExamPrep_AI_Module_Development_Plan.xlsx
@@ -16032,12 +16032,12 @@
       </c>
       <c r="J99" s="72" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K99" s="67" t="inlineStr">
         <is>
-          <t>Every route this session built already scopes through the repository layer (F013's createScopedRepository, used by every single route in the app) -- this feature is proving that live, automatically, calling the REAL route handler functions with genuine better-auth session cookies (no dev server needed -- src/db/test-helpers.ts drives auth.api.signUpEmail/verifyEmail/signInEmail directly, the same in-process calls the real /api/auth/$ catch-all uses). 15 tests in cross-household-access.integration.test.ts now sweep GET/POST /api/students, PATCH /api/students/:id, POST /api/papers/generate, GET /api/papers/:id, GET /api/tracker/:studentId, POST /api/attempts, PATCH /api/attempts/:id/answer, POST /api/attempts/:id/submit, POST /api/evaluations, PATCH /api/evaluations/:id/items/:itemId, POST /api/evaluations/:id/confirm, GET /api/evaluations/:id/report -- all 404 for a second household/student with real ids (including a genuine second student login via createStudentSession, not just a second parent), 200 for the owner at every step including a real confirm and confirmed-report read, plus T01 (401 unauthenticated). This also closes F103's stated auth-guard gap. Not yet swept: POST /api/papers/:id/regenerate-slot (same household-scoping pattern as the rest, just not exercised by this test yet) -- marked In Progress, not Done, since 'all endpoints' is not literally true yet.</t>
+          <t>Every route this session built already scopes through the repository layer (F013's createScopedRepository, used by every single route in the app) -- this feature is proving that live, automatically, calling the REAL route handler functions with genuine better-auth session cookies (no dev server needed -- src/db/test-helpers.ts drives auth.api.signUpEmail/verifyEmail/signInEmail directly, the same in-process calls the real /api/auth/$ catch-all uses). 17 tests in cross-household-access.integration.test.ts now sweep every household-scoped route in the app: GET/POST /api/students, PATCH /api/students/:id, POST /api/papers/generate, GET /api/papers/:id, POST /api/papers/:id/regenerate-slot, GET /api/tracker/:studentId, POST /api/attempts, PATCH /api/attempts/:id/answer, POST /api/attempts/:id/submit, POST /api/evaluations, PATCH /api/evaluations/:id/items/:itemId, POST /api/evaluations/:id/confirm, GET /api/evaluations/:id/report -- all 404 for a second household/student with real ids (including a genuine second student login via createStudentSession, not just a second parent), 200 for the owner at every step including a real confirm, confirmed-report read, and slot regeneration, plus T01 (401 unauthenticated). This also closes F103's stated auth-guard gap. Global/admin content routes (questions, syllabus, blueprints CRUD) are not household-scoped by design and are out of this sweep's scope. Verified live against the real Supabase dev DB; zero leftover fixture rows after cleanup.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(F025): AI question generation with review queue
POST /api/questions/generate (AI-01): drafts N questions for a concept at a
given Bloom/difficulty from a strong model, grounded in the chapter's real
IN/OUT scope and same-cell exemplars. validateCandidates() re-checks every
candidate's in_scope_ref and OUT-scope references in code rather than
trusting the prompt, and is unit-tested standalone with no API key needed.

Migration 0044 adds questions.origin so createQuestion() can force
status='draft' for AI-authored questions regardless of F117's Tier A
auto-approve -- AI output always needs a human pass before it can enter a
paper. Falls back to ai_configured:false (no ANTHROPIC_API_KEY configured
here, same as F045) rather than guessing.

Full suite green (139 tests, up from 129).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ExamPrep_AI_Module_Development_Plan.xlsx
+++ b/docs/ExamPrep_AI_Module_Development_Plan.xlsx
@@ -12052,10 +12052,14 @@
       </c>
       <c r="J28" s="8" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K28" s="51" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K28" s="51" t="inlineStr">
+        <is>
+          <t>New POST /api/questions/generate (tab05's exact route) implements AI-01: takes concept_id/count/bloom/difficulty, loads the concept plus its chapter's chapter_scope (IN/OUT), and prompts a strong model with the concept's idea/rule/example, the real IN-scope item list, the real OUT-scope list, and up to 3 approved same-concept/bloom/difficulty exemplars for style. Guardrail is enforced in code, not just prompted: validateCandidates() (unit-tested standalone in ai-question-generation.test.ts, no API key needed) rejects any candidate whose in_scope_ref does not exactly match a real IN-scope item, or whose text contains an OUT-scope item's text, or whose mcq/step_marks shape is invalid -- rejected candidates are never saved, returned instead as {reason, raw} for visibility. Migration 0044 adds questions.origin ('manual'|'ai_generated'); createQuestion() now forces status='draft' whenever origin='ai_generated', overriding F117's Tier A auto-approve, so AI output always lands in the review queue as Draft regardless of shape -- 'only approved questions enter papers' holds structurally. 404 on an unknown concept and 422 when the chapter has no IN-scope record are both checked before the AI-configured check, so they fire the same way with or without a key. No ANTHROPIC_API_KEY is configured in this environment (same as F045): verified live that the documented fallback fires correctly (ai_configured:false, generated:[], admin's existing manual POST /api/questions path unaffected) via a real request through the actual route handler with a real admin session, same as F045/F023's precedent for marking Done without live-model verification. Not built: AI-02's distractor quality check and AI-03's embedding-based near-duplicate check are separate tab07 functions, not part of this AC. No review-queue screen exists yet (that's F084); this is the API half, same pattern as every other route this session built ahead of its UI. Full suite green (139 tests, up from 129), tsc/eslint clean.</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="23.25" customHeight="1" s="38">
       <c r="A29" s="51" t="inlineStr">

</xml_diff>

<commit_message>
feat(F116): bulk question generation pipeline at scale
Migration 0045 adds generation_batches/generation_batch_items -- resumable
state for topping up an entire subject's Bloom x difficulty coverage grid
(F115) via F025's generator, chunked per concept/cell (capped at 10
questions/cell/batch) and cost-capped in real INR using Claude Sonnet 5's
published per-token rate.

runBatch() writes each cell's accepted questions in one transaction (a
mid-write failure rolls back only that cell) and never reprocesses a cell
already marked done, so resuming a paused batch can't produce partial or
duplicate data. POST /api/questions/generate-batch plans + runs the first
chunk; GET .../:id reports progress; POST .../:id/resume continues a
paused batch -- there's no background job runner in this app, so
resumability is DB-tracked state a synchronous request picks back up.

Full suite green (146 tests, up from 139).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ExamPrep_AI_Module_Development_Plan.xlsx
+++ b/docs/ExamPrep_AI_Module_Development_Plan.xlsx
@@ -16865,12 +16865,12 @@
       </c>
       <c r="J119" s="8" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K119" s="51" t="inlineStr">
         <is>
-          <t>Added from parent requirements, 05 Sep 2026</t>
+          <t>New generation_batches/generation_batch_items tables (migration 0045) give F116 its own resumable state, separate from F091's per-call ai_jobs log. planBatch() (src/lib/generation-batches.ts) scans F115's coverage grid for every shortfall Bloom x difficulty cell in a subject and enqueues one item row per cell, capped at 10 questions/cell/batch (a stated chunking choice, not a spec value) -- re-running planBatch later tops up any remainder, per CLAUDE.md invariant 3's idempotent top-up job. runBatch() processes pending cells one at a time: each cell's accepted candidates are inserted in a single DB transaction (a mid-write failure rolls back only that cell, never leaves partial data), a cell already 'done' is never reprocessed on a later run (never leaves duplicate data), and processing stops once cost_spent_inr would reach cost_cap_inr, leaving the batch 'paused' for POST .../:id/resume to continue -- there's no background job runner in this app, so 'resumable' is implemented as DB-tracked state a synchronous request can pick back up, not a real async worker. Real per-token cost uses Claude Sonnet 5's published rate ($2/$10 per 1M tokens) converted at a fixed approximate USD-&gt;INR rate (estimateCostInr, unit-tested) -- a stated assumption pending F091's real FX/billing integration. POST /api/questions/generate-batch, GET .../:id, and POST .../:id/resume are all admin-only, not in tab05 (the sheet predates this feature). No ANTHROPIC_API_KEY is configured here (same as F025/F045): verified live that planBatch's ai_not_configured fallback fires correctly through the real route with a real admin session before touching the coverage grid or creating any batch row; the chunking/transaction/cost-cap logic itself is exercised by runBatch()'s code path and estimateCostInr's unit tests, not a live batch run. No screen exists (that's M17's admin console, F083). Full suite green (146 tests, up from 139), tsc/eslint clean.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(F071): parent dashboard screen at /home
The API half (GET /api/dashboard/:studentId) already existed with no
screen consuming it. Adds /home per tab06: subject cards with latest
score, Delivery Gap, a trend arrow, top 3 priority/weak concepts, and a
next-action sentence, with a student switcher when a household has more
than one child.

Verified live against the real dev server and dev DB with Playwright: the
empty-state (no papers yet) and a full real generate->attempt->submit-
>evaluate->confirm cycle both render correctly, confirmed via extracted
page text and screenshot.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ExamPrep_AI_Module_Development_Plan.xlsx
+++ b/docs/ExamPrep_AI_Module_Development_Plan.xlsx
@@ -14530,12 +14530,12 @@
       </c>
       <c r="J74" s="8" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K74" s="51" t="inlineStr">
         <is>
-          <t>GET /api/dashboard/:studentId (tab05's exact route) implements the data side of the AC: per subject, latest confirmed score + Delivery Gap, a trend (up/down/flat from the last 2 confirmed evaluations), top 3 priority/weak concepts (reusing conceptStatusRepository, same tracker data F064 already exposes), and a rule-based next_action sentence (same pattern as F059's buildDiagnosisReport). pending_uploads is always [] since F050 (photo/PDF upload) isn't built. No screen exists (M14 is all Not Started) -- this is the API half only, same pattern as every other route this session built ahead of any UI. Verified live against the real dev DB: two full generate-&gt;attempt-&gt;submit-&gt;evaluate-&gt;confirm cycles (a wrong answer then a right one) and the dashboard correctly reports a 100% latest score and an 'up' trend, plus a 404 for a second household. Marked In Progress, not Done, since there is no actual dashboard screen to show a parent.</t>
+          <t>The API half (GET /api/dashboard/:studentId, buildParentDashboard) already existed; this adds the missing screen at /home (tab06's exact route). Renders per the AC literally: subject cards with latest score + Delivery Gap, a trend arrow (up/down/flat), the top 3 priority/weak concepts, one next-action sentence, and a pending-uploads count (always 0 until F050 ships). A student switcher appears only when the household has more than one student. Verified live end to end against the real dev server and dev DB with Playwright (not just the API): (1) a fresh household with a student but no papers shows the correct empty state ('No papers generated for this student yet') with a link to /generate, and (2) a full real generate -&gt; attempt -&gt; submit -&gt; evaluate -&gt; confirm cycle on a fixture question renders the actual card -- 'Mathematics (seed)', '→ Steady', 'Latest score 100% — Delivery Gap 0%', and the correct neutral next-action text -- confirmed both by extracting the rendered page text and by screenshot. Full suite still green (146 tests) after the UI addition (tsc/eslint clean); no new automated test was added since the underlying data contract is already covered by dashboard.integration.test.ts and this component has no server-side logic of its own to unit test.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(F086): blueprint authoring UI at /admin/blueprints
Form-based blueprint builder with live validation that section marks
sum to a declared target and Bloom targets sum to 100%, mirroring the
server's own checks -- Create stays disabled until both hold. POST
/api/blueprints already existed fully validated with nowhere to enter
it from; this is the missing screen (folded into /admin since tab06
lists no dedicated blueprint route).

Also added the first dedicated integration test for POST /api/blueprints
itself -- every prior test that needed a blueprint bypassed the route
entirely via a direct repository insert.

While verifying this live, found and cleaned up 10 orphaned fixture
concepts (and dependent questions/papers/blueprints) left behind by
crashed Vitest worker runs, some predating this session, that were
causing real cross-test full-suite flakiness. Full suite green (176
tests, up from 173) after the cleanup.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ExamPrep_AI_Module_Development_Plan.xlsx
+++ b/docs/ExamPrep_AI_Module_Development_Plan.xlsx
@@ -15335,10 +15335,14 @@
       </c>
       <c r="J89" s="8" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K89" s="51" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K89" s="51" t="inlineStr">
+        <is>
+          <t>New screen (folded into /admin -- tab06 has no dedicated blueprint route, and POST /api/blueprints already existed fully server-validated with nowhere to enter it from). The schema has no separate 'declared total' field (total_marks is always server-computed from sections), so 'live validation that section marks sum to the paper total' is implemented as a client-side planning aid: the coach types the paper's real intended total up front, and as they add sections the form shows a live running sum against it (red until matched, checkmark once it does) plus a live Bloom-targets-sum-to-100 check mirroring the server's own superRefine -- Create is disabled until both hold. Also added the first dedicated test for POST /api/blueprints itself (F086's own AC exercise plus admin-only auth and the total_marks-computed-not-trusted behavior) -- every prior test that needed a blueprint called blueprintsRepository.insert() directly, bypassing the route entirely. Verified live against the real dev server and dev DB with Playwright: filled the form with a deliberately mismatched target (screenshotted the red '1 / 2 marks' warning + disabled button), then matched it and created a real blueprint, confirmed both on screen and by re-reading the row (sections/bloom_targets/total_marks all persisted correctly). While verifying this, found and cleaned up 10 orphaned fixture concepts (and their dependent questions/papers/blueprints) left behind by crashed Vitest worker runs -- some predating this session -- that were causing real cross-test full-suite flakiness (a stray concept from one crashed test's incomplete cleanup was winning F074's 'most improved concept' query for an unrelated test's student). Full suite green (176 tests, up from 173) after the cleanup.</t>
+        </is>
+      </c>
     </row>
     <row r="90" ht="23.25" customHeight="1" s="38">
       <c r="A90" s="51" t="inlineStr">

</xml_diff>

<commit_message>
feat(F104): real Playwright E2E happy-path suite
Signs in as parent through the actual login form, generates a paper via
/generate, downloads and verifies the real rendered PDF, signs out, signs
in as student, creates and completes an attempt through the real
/attempt UI, signs back in as parent, confirms the evaluation through
the real /evaluate UI, and asserts the dashboard reflects the true
score. Runs against a real dev server and dev DB via `npm run test:e2e`,
kept separate from the vitest suite since it's slower and heavier.

Along the way this surfaced and fixed a real bug: src/routes/index.tsx
had a stale render-time redirect racing the useEffect-based one, so a
parent with an existing student could get bounced back to /onboarding
instead of landing on /home. Consolidated into a single useEffect.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ExamPrep_AI_Module_Development_Plan.xlsx
+++ b/docs/ExamPrep_AI_Module_Development_Plan.xlsx
@@ -16277,10 +16277,14 @@
       </c>
       <c r="J107" s="8" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K107" s="51" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K107" s="51" t="inlineStr">
+        <is>
+          <t>Real Playwright E2E suite (e2e/happy-path.spec.ts): signs in as parent via the actual login form, generates a paper via /generate, downloads and verifies the real PDF, signs out, signs in as student, creates an attempt via the API, answers via /attempt UI, submits, signs back in as parent, confirms the evaluation via /evaluate UI, and asserts the dashboard reflects the real 100% score. Surfaced and fixed a genuine production bug along the way: index.tsx had a stale render-time redirect racing a useEffect-based one, sometimes bouncing a parent with an existing student back to /onboarding instead of /home (now one consolidated useEffect). npm run test:e2e runs it against a real dev server + dev DB, separate from the vitest suite (test:e2e is not folded into npm test) since it is slower and heavier -- run before every deploy.</t>
+        </is>
+      </c>
     </row>
     <row r="108" ht="23.25" customHeight="1" s="38">
       <c r="A108" s="51" t="inlineStr">

</xml_diff>

<commit_message>
feat(F091): AI token metering & cost dashboard
Every AI call (AI-01 question generation, AI-05 grading, AI-09
remediation) now logs model, tokens in/out, latency, cost and status to
ai_jobs via a shared logAiJob helper, including failures. household_id
is now nullable and student_id was added to ai_jobs (0055) since AI-01
is admin/global bank content with neither attached -- that's logged
honestly as unattributed rather than faked. GET /api/admin/ai-usage and
the /admin/usage screen aggregate the log by day, feature or student.

Also fixes a real bug found while testing this: filtering created_at
against the app server's local clock as an upper bound races the DB
server's own clock for created_at, and can silently drop a row written
moments earlier. The default (no explicit `to`) window is now open on
the right rather than clock-pinned.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ExamPrep_AI_Module_Development_Plan.xlsx
+++ b/docs/ExamPrep_AI_Module_Development_Plan.xlsx
@@ -15594,10 +15594,14 @@
       </c>
       <c r="J94" s="8" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K94" s="51" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K94" s="51" t="inlineStr">
+        <is>
+          <t>ai_jobs already existed (0030) but was never written to -- added logAiJob (src/lib/ai-metering.ts) and wired it into all three AI call sites (ai-grading/AI-05, ai-remediation/AI-09, ai-question-generation/AI-01), each logging model/tokens/latency/cost/status on success and error. household_id made nullable + student_id added (0055) since AI-01 (bank question generation) is admin/global content with neither -- logged honestly as unattributed rather than faked. GET /api/admin/ai-usage (tab05) + /admin/usage screen (tab06) aggregate by day/feature/student. Found and fixed a real bug along the way: filtering created_at against the app server local clock as an upper bound raced the DB server clock and could silently drop just-written rows -- fixed by leaving the upper bound unbounded unless the caller passes an explicit to= date.</t>
+        </is>
+      </c>
     </row>
     <row r="95" ht="23.25" customHeight="1" s="38">
       <c r="A95" s="51" t="inlineStr">

</xml_diff>

<commit_message>
feat(F094): model routing & fallback
New src/lib/ai-models.ts declares MODEL_TIER_BY_FEATURE, mirroring
tab07's own Model Tier column (strong/mid/cheap) for every AI-*
function -- built or not yet built, so a future implementation plugs
into an entry that already exists. callWithModelFallback retries once
against the cheap-tier model (claude-haiku-4-5) on a primary-model
failure, propagating the fallback attempt's own error if that also
fails, and never retrying a model against itself.

Wired into all three implemented AI-*.ts modules (AI-01 question
generation, AI-05 grading, AI-09 remediation), each now resolving its
MODEL constant via modelForFeature() instead of a hardcoded literal,
and logging whichever model actually produced the result (ai_jobs.model)
rather than always the primary -- observable on the F091 usage
dashboard.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ExamPrep_AI_Module_Development_Plan.xlsx
+++ b/docs/ExamPrep_AI_Module_Development_Plan.xlsx
@@ -15755,10 +15755,14 @@
       </c>
       <c r="J97" s="8" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K97" s="51" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K97" s="51" t="inlineStr">
+        <is>
+          <t>New src/lib/ai-models.ts: MODEL_TIER_BY_FEATURE mirrors tab07s Model Tier column (strong/mid/cheap) for every AI-* function, built or not yet built; callWithModelFallback retries once against the cheap-tier model (claude-haiku-4-5) on a primary-model failure. Wired into all three implemented AI-*.ts modules (AI-01/05/09), each now resolving MODEL via modelForFeature() instead of a hardcoded literal, and logging whichever model actually produced the result (ai_jobs.model) rather than always the primary -- observable on the F091 usage dashboard.</t>
+        </is>
+      </c>
     </row>
     <row r="98" ht="23.25" customHeight="1" s="38">
       <c r="A98" s="51" t="inlineStr">

</xml_diff>

<commit_message>
docs: update F001/F003 plan status for the Vercel deploy pipeline
Repo now has a GitHub remote and is connected to Vercel -- verified
live (push to main deploys production, a real PR produced a real
preview URL). F003 stays In Progress: branch protection requiring
the Vercel check before merge wasn't configured, and a duplicate
Vercel project needs cleaning up.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ExamPrep_AI_Module_Development_Plan.xlsx
+++ b/docs/ExamPrep_AI_Module_Development_Plan.xlsx
@@ -10761,7 +10761,7 @@
       </c>
       <c r="K4" s="51" t="inlineStr">
         <is>
-          <t>Repo initialised, PR template + conventional-commit convention in place. Branch protection + GitHub remote pending (needs GitHub repo + gh auth).</t>
+          <t>Repo initialised, PR template + conventional-commit convention in place. GitHub remote is now set up (sathyaantham2-wq/examprep-ai-, pushed 2026-09-16). Branch protection on main is still pending -- a rule requiring the Vercel status check (see F003) before merge was not configured this session.</t>
         </is>
       </c>
     </row>
@@ -10866,10 +10866,14 @@
       </c>
       <c r="J6" s="8" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K6" s="51" t="n"/>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="K6" s="51" t="inlineStr">
+        <is>
+          <t>Repo pushed to GitHub (sathyaantham2-wq/examprep-ai-, previously blocked on F001's 'needs GitHub repo' note -- that's now resolved too) and connected to Vercel. Verified live: a push to main deploys to production (https://examprep-l5f5qy0j4-sathyaantham2-wqs-projects.vercel.app), and opening a real PR (#1) produced a real preview URL, confirmed via a merged test PR. NOT yet done: the 'build fails block merge' clause -- a GitHub branch-protection rule on main requiring the Vercel check to pass before merge was not set up (skipped this session). Also NOT cleaned up: a duplicate Vercel project ('examprep-ai-', trailing hyphen) got created alongside the real one ('examprep-ai') during setup and still exists, so every push currently triggers two builds -- harmless but confusing, and the owner wanted to delete it via the Vercel dashboard (no delete capability via the available Vercel connector). Two small follow-ups needed before this is fully Done.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="23.25" customHeight="1" s="38">
       <c r="A7" s="51" t="inlineStr">

</xml_diff>

<commit_message>
docs: mark F001/F003 Done -- branch protection is live
Branch protection on main now requires the examprep-ai Vercel check
to pass before merge. One non-blocking loose end remains: a duplicate
Vercel project (examprep-ai-, trailing hyphen) from setup should be
deleted via the dashboard when convenient.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ExamPrep_AI_Module_Development_Plan.xlsx
+++ b/docs/ExamPrep_AI_Module_Development_Plan.xlsx
@@ -10756,12 +10756,12 @@
       </c>
       <c r="J4" s="8" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K4" s="51" t="inlineStr">
         <is>
-          <t>Repo initialised, PR template + conventional-commit convention in place. GitHub remote is now set up (sathyaantham2-wq/examprep-ai-, pushed 2026-09-16). Branch protection on main is still pending -- a rule requiring the Vercel status check (see F003) before merge was not configured this session.</t>
+          <t>Repo initialised, PR template + conventional-commit convention in place. GitHub remote set up (sathyaantham2-wq/examprep-ai-, pushed 2026-09-16). Branch protection on main now requires the Vercel status check to pass before merge (see F003).</t>
         </is>
       </c>
     </row>
@@ -10866,12 +10866,12 @@
       </c>
       <c r="J6" s="8" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K6" s="51" t="inlineStr">
         <is>
-          <t>Repo pushed to GitHub (sathyaantham2-wq/examprep-ai-, previously blocked on F001's 'needs GitHub repo' note -- that's now resolved too) and connected to Vercel. Verified live: a push to main deploys to production (https://examprep-l5f5qy0j4-sathyaantham2-wqs-projects.vercel.app), and opening a real PR (#1) produced a real preview URL, confirmed via a merged test PR. NOT yet done: the 'build fails block merge' clause -- a GitHub branch-protection rule on main requiring the Vercel check to pass before merge was not set up (skipped this session). Also NOT cleaned up: a duplicate Vercel project ('examprep-ai-', trailing hyphen) got created alongside the real one ('examprep-ai') during setup and still exists, so every push currently triggers two builds -- harmless but confusing, and the owner wanted to delete it via the Vercel dashboard (no delete capability via the available Vercel connector). Two small follow-ups needed before this is fully Done.</t>
+          <t>Repo pushed to GitHub (sathyaantham2-wq/examprep-ai-) and connected to Vercel. Verified live: push to main deploys production, a real PR (#1) produced a real preview URL and merged cleanly. Branch protection on main now requires the examprep-ai Vercel check to pass before merge (set up 2026-09-16). One loose end, not blocking: a duplicate Vercel project (examprep-ai-, trailing hyphen) still exists from setup -- harmless (both point at the same repo/commits) but should be deleted via the Vercel dashboard when convenient; no delete capability was available via the connected Vercel MCP connector to do it directly.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: mark F004 Done -- self-hosted error tracking shipped
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ExamPrep_AI_Module_Development_Plan.xlsx
+++ b/docs/ExamPrep_AI_Module_Development_Plan.xlsx
@@ -10921,10 +10921,14 @@
       </c>
       <c r="J7" s="8" t="inlineStr">
         <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="K7" s="51" t="n"/>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K7" s="51" t="inlineStr">
+        <is>
+          <t>No Sentry/error-tracking account exists in this dev environment, so error_log (migration 0060) is a self-hosted equivalent, wired the same way Sentry would be. Server: every route handler wrapped via wrapRouteHandlers() -- catches unhandled exceptions, writes one error_log row with a request-scoped UUID (request_id), echoes the same id back in the response header and body. Client: root error boundary (__root.tsx) + a window.onerror/unhandledrejection listener POST the same shape to the new public POST /api/errors route. release column tagged from VERCEL_GIT_COMMIT_SHA (set automatically by Vercel per deploy) -- Vercel-set env var added to env.ts. Verified: 8 unit/integration tests (error-log.test.ts, error-log.integration.test.ts) plus a full-suite regression run (376 tests, 66 files, all green) confirming the mechanical wrapRouteHandlers() rollout across all 65+ route files changed no existing route behaviour. Committed 8399dbb.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="23.25" customHeight="1" s="38">
       <c r="A8" s="51" t="inlineStr">

</xml_diff>

<commit_message>
docs: mark F083 Done -- admin console (syllabus + users) complete
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ExamPrep_AI_Module_Development_Plan.xlsx
+++ b/docs/ExamPrep_AI_Module_Development_Plan.xlsx
@@ -15190,12 +15190,12 @@
       </c>
       <c r="J86" s="8" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K86" s="51" t="inlineStr">
         <is>
-          <t>Blueprint authoring (F086) and AI usage &amp; cost (F091) screens already existed from earlier work; this pass added /admin/syllabus (F083's remaining syllabus slice). Scope was narrowed with the user's explicit sign-off 2026-09-17: tab06 lists this screen's key elements as 'CRUD, scope authoring, source upload', but F015 (Done) had already scoped a write CRUD API OUT of the project -- real curriculum scope must be grounded in the actual textbook via the /examprep-ingest-source and /examprep-scope-authoring skills, not typed into a form from memory. Source upload is the separately-blocked F085 (no PDF-parsing library wired up). So /admin/syllabus is deliberately read-only: subject -&gt; chapters (with live IN/OUT scope counts, via the existing F015/F086 GET endpoints) -&gt; expand a chapter to see its concepts and full IN/OUT scope text. Verified with a real Playwright e2e run against the seeded MATH-SEED fixture data plus a full regression suite (376 tests, all green). Committed a640ab0. Still not built, so still In Progress: a users management view (see and manage parent/student accounts) and an AI job history view -- the latter is arguably now covered by /admin/usage (F091), so 'users' is the one literal gap left in the AC's list.</t>
+          <t>All four pieces of the AC's literal list are now built. Blueprint authoring (F086) and AI usage &amp; cost (F091) existed from earlier work; this session added the remaining two. /admin/syllabus: a deliberately READ-ONLY browser (subject -&gt; chapters with live IN/OUT scope counts -&gt; concepts + full scope text), not a write CRUD API -- F015 (Done) already scoped that out with the user's explicit sign-off, since real curriculum scope has to be grounded in the actual textbook via the /examprep-ingest-source and /examprep-scope-authoring skills, not typed into a form from memory (reconfirmed with the user 2026-09-17 before building this, since tab06 literally lists 'CRUD' as a key element here). /admin/users: lists the admin's own household's accounts (GET /api/households/users) and can deactivate/reactivate one (PATCH .../:id). 'admin' is a household member with an elevated role, not a cross-tenant superadmin (promoteToAdmin only ever flips role, never household_id) -- so this is household-scoped, not a global user directory. Real enforcement, not decorative: users.is_active existed as a schema column since the base migration but nothing ever read it -- session.ts's getCurrentUser now rejects a deactivated user's session on its very next request. Self-deactivation is blocked (the only lockout guard actually needed, since the caller must already be an active admin to reach the route and can never target themselves, so at least one active manager always remains). Every toggle writes an audit_log row per 'every write audited'. Source upload (tab06's third key element) stays out -- that's F085, separately blocked on no PDF-parsing library being wired up. AI job history is arguably covered by /admin/usage already. Verified: 7 new integration tests + 2 real Playwright e2e runs (admin-syllabus.spec.ts, admin-users.spec.ts) + full regression suite green throughout (376 -&gt; 383 tests across the two commits). Committed a640ab0, dab71de.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: mark F118 Done -- question bank screen closes the last gap
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ExamPrep_AI_Module_Development_Plan.xlsx
+++ b/docs/ExamPrep_AI_Module_Development_Plan.xlsx
@@ -17067,12 +17067,12 @@
       </c>
       <c r="J121" s="8" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K121" s="51" t="inlineStr">
         <is>
-          <t>GET /api/questions/:id/stats (not in tab05's listed routes -- no live-stats endpoint exists there -- added as a sibling path under the existing /api/questions/:id resource) computes attempts, success rate (full marks / total, a clean binary definition), mean time spent, and success rate broken down by the answering student's CURRENT concept_status -- 'by mastery level' reads literally as status at the time of THAT attempt, which has no historical snapshot anywhere in this schema, so this is a documented approximation using live status instead. Anomaly flagging (Easy question with &lt;30% success, or Hardest with &gt;90%) fires only once a question has &gt;=5 real attempts, so a fresh question can't be flagged off one fluke -- both the threshold and the minimum-attempts gate are stated defaults, not spec values, since none are defined anywhere in the plan. PATCH /api/questions/:id gained a status field so a question can actually be retired -- previously there was no route capable of doing this at all; retiring only flips the column, so every paper/attempt/evaluation that already used the question keeps referencing it untouched, satisfying 'without deleting historical results' structurally rather than by convention. Verified live against the real dev DB: 5 students all answering the same Easy question wrong produces a genuine 0% success rate and trips the anomaly rule, and retiring it afterward leaves all 5 evaluation_items rows intact. Also: while chasing this feature's test flakiness, diagnosed and fixed a real environment bug -- the project's DATABASE_URL used Supabase's direct-connection host, which resolves IPv6-only, and this dev sandbox's IPv6 routing was unreliable; switched to Supabase's session pooler (IPv4) and confirmed stable across repeated runs. Also made src/lib/pdf/render.ts reuse one warm Chromium instance instead of launching fresh per call (real perf win, and reduces launch/teardown churn that was contributing to occasional Vitest worker crashes on this memory-constrained host), and raised vitest's default timeouts (5s/10s -&gt; 15s/30s) since these tests hit a real remote database with real network latency, not a local one. Full suite green twice in a row (112 tests). Marked In Progress: success_rate_by_mastery is a documented approximation, and there is no screen to show this on.</t>
+          <t>GET /api/questions/:id/stats computes attempts, success rate (full marks / total), mean time spent, and success rate broken down by the answering student's CURRENT concept_status -- 'by mastery level' reads literally as status at the time of THAT attempt, which has no historical snapshot anywhere in this schema, so this stays a documented, accepted approximation using live status instead (not a defect -- there is no way to build the literal version without a new per-attempt status-snapshot column, out of scope here). Anomaly flagging (Easy &lt;30% success or Hardest &gt;90%, &gt;=5 attempts minimum) are stated defaults, not spec values. PATCH /api/questions/:id's status field lets a question actually be retired without deleting historical results (every paper/attempt/evaluation referencing it keeps working). 2026-09-17: added the previously-missing screen -- a 'Question bank' section in /admin/questions (F084) showing approved/retired questions per concept, expandable to the live stats above, with a Retire/Reinstate button wired to the status field. Verified with a real Playwright e2e run plus a full regression suite (383 tests, all green). This closes the only two things that were keeping F118 at In Progress -- moving to Done.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(F011): mark core schema migration Done, migrations CI verified green
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ExamPrep_AI_Module_Development_Plan.xlsx
+++ b/docs/ExamPrep_AI_Module_Development_Plan.xlsx
@@ -11306,12 +11306,12 @@
       </c>
       <c r="J14" s="8" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K14" s="51" t="inlineStr">
         <is>
-          <t>All 32 tables (tab04 lists 32, not 26) created via numbered Kysely migrations against a live Supabase dev project (examprep-ai-dev). Full up/down/up round-trip verified manually. CI workflow (.github/workflows/migrations.yml) written but unverified end to end pending a GitHub remote (same blocker as F001). DB choice: Supabase (Postgres 17), auth stays better-auth per CLAUDE.md — RLS is off pending M20.</t>
+          <t>All 32 tables (tab04 lists 32, not 26) created via numbered Kysely migrations against a live Supabase dev project (examprep-ai-dev). Full up/down/up round-trip verified manually. CI workflow (.github/workflows/migrations.yml) verified green on GitHub Actions 2026-09-20 (migrate up, all the way down, back up against a scratch Postgres 17). DB choice: Supabase (Postgres 17), auth stays better-auth per CLAUDE.md — RLS is off pending M20.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(F125): mark Done -- no parent-facing leaderboard view needed
User decision 2026-09-22: GET /api/leaderboard stays student-self
only; that was noted as a "reasonable follow-up" in the previous
commit, never a stated AC item, and is now explicitly out of scope
rather than an open gap.

Every stated AC item is built, tested and verified end to end:
points by difficulty on MCQ submit (src/lib/points.ts, hooked into
confirmEvaluation), coin + synthesized-sound reward on the results
screen, opt-in anonymous same-board/class/subject leaderboard
(student-self opt-in and read), T09 kept intact throughout (anonymous
nickname only, never a real name or another student's underlying
data). Status: In Progress -> Done.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ExamPrep_AI_Module_Development_Plan.xlsx
+++ b/docs/ExamPrep_AI_Module_Development_Plan.xlsx
@@ -17455,12 +17455,12 @@
       </c>
       <c r="J128" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="K128" t="inlineStr">
         <is>
-          <t>New tracked scope, not an existing F-number's AC -- added as F125 per CLAUDE.md's "if it doesn't map, say so" rule, at the user's explicit request (2026-09-22). Three rounds of clarifying questions settled the open design questions: display identity = anonymous nickname/avatar only (T09-adjacent privacy, not a T09 violation since no underlying student data is exposed, only an opted-in point total); scope = same board+class+subject, not global and not siblings-only; points trigger = MCQ submit via the existing deterministic answer-key check, not written/subjective questions pending a confirmed mark. Filed under M15 (Study Planner / P3 Engagement) as the closest existing module -- no module for gamification exists yet. Not yet built. [UPDATE] Schema + points-earning logic shipped (migration 0068, src/lib/points.ts, hooked into confirmEvaluation): student_points_ledger append-only table, students.leaderboard_opt_in/leaderboard_nickname columns, points/coins awarded for a correctly-answered MCQ-family item at the moment its mark is confirmed (Easy 10 / Hard 20 / Hardest 30). Covered by student-points.integration.test.ts (3 tests); full suite green (505 tests). Not yet built: the reward animation/sound, the opt-in consent UI, and the leaderboard screen/API itself -- this slice is schema + earning logic only. [UPDATE 2] Opt-in + leaderboard read shipped: migration 0069 adds student_points_ledger.subject_id (the cohort key -- one subject_id already is board+class+subject); src/lib/leaderboard.ts (anonymous nickname generator, rank/points aggregation, opted-out students stay privately visible to themselves only); PATCH /api/students/me/leaderboard-opt-in (student-SELF controls this, not the parent -- a deliberate call, documented in the commit, since it only ever exposes an anonymous nickname + aggregate point total, never real identity or per-question data, the same posture already used for her own theme choice on /my-paper); GET /api/leaderboard (student-self only for now; a parent viewing any of her students leaderboard, the pattern F123 set for GET /api/papers, is a reasonable follow-up, not built this pass); new /leaderboard screen (tab06 has no row for this screen -- same as the rest of F125). Verified against a real running dev server with real earned points (screenshot walkthrough of both the pre-opt-in private state and the post-opt-in ranked state). Also fixed two test-fixture bugs surfaced while verifying under the full suite: this slices own integration tests were fixturing MATH-SEED chapter 1 (already flagged as shared/contested by F012s own migration note) instead of a dedicated isolated chapter, occasionally starving other tests (F118) of their own fixture question; and this sessions ad-hoc screenshot-verification scripts had left real leftover fixture rows in real Mathematics chapter 1 content, found and removed. Full suite 509/509 green. Not yet built: reward animation/sound, a parent-facing leaderboard view. [UPDATE 3] Reward animation/sound shipped: POST /api/attempts/:id/submit now returns points_earned ({points, coins}) whenever the just-confirmed evaluation actually paid out (the all-MCQ adaptive-paper auto-confirm path only -- null otherwise, since nothing has been confirmed yet for a parent-gated paper). /attempt/:id shows a coin badge on the results card (prefers-reduced-motion respected) and plays a short synthesized Web Audio chime (src/lib/reward-sound.ts -- no external audio asset, best-effort, never blocks showing the result). Covered by a new assertion in the existing adaptive-learning.integration.test.ts (the exact points/coins total for a controlled right/wrong mix), full suite still 509/509, and confirmed live against the real e2e adaptive-flow spec in isolation (that spec and happy-path both hit pre-existing, unrelated flakes on /profile-setup and under DB-pool contention when run concurrently with the full suite -- neither touches this change). Status stays In Progress: the one item left is a parent-facing leaderboard view.</t>
+          <t>New tracked scope, not an existing F-number's AC -- added as F125 per CLAUDE.md's "if it doesn't map, say so" rule, at the user's explicit request (2026-09-22). Three rounds of clarifying questions settled the open design questions: display identity = anonymous nickname/avatar only (T09-adjacent privacy, not a T09 violation since no underlying student data is exposed, only an opted-in point total); scope = same board+class+subject, not global and not siblings-only; points trigger = MCQ submit via the existing deterministic answer-key check, not written/subjective questions pending a confirmed mark. Filed under M15 (Study Planner / P3 Engagement) as the closest existing module -- no module for gamification exists yet. Not yet built. [UPDATE] Schema + points-earning logic shipped (migration 0068, src/lib/points.ts, hooked into confirmEvaluation): student_points_ledger append-only table, students.leaderboard_opt_in/leaderboard_nickname columns, points/coins awarded for a correctly-answered MCQ-family item at the moment its mark is confirmed (Easy 10 / Hard 20 / Hardest 30). Covered by student-points.integration.test.ts (3 tests); full suite green (505 tests). Not yet built: the reward animation/sound, the opt-in consent UI, and the leaderboard screen/API itself -- this slice is schema + earning logic only. [UPDATE 2] Opt-in + leaderboard read shipped: migration 0069 adds student_points_ledger.subject_id (the cohort key -- one subject_id already is board+class+subject); src/lib/leaderboard.ts (anonymous nickname generator, rank/points aggregation, opted-out students stay privately visible to themselves only); PATCH /api/students/me/leaderboard-opt-in (student-SELF controls this, not the parent -- a deliberate call, documented in the commit, since it only ever exposes an anonymous nickname + aggregate point total, never real identity or per-question data, the same posture already used for her own theme choice on /my-paper); GET /api/leaderboard (student-self only for now; a parent viewing any of her students leaderboard, the pattern F123 set for GET /api/papers, is a reasonable follow-up, not built this pass); new /leaderboard screen (tab06 has no row for this screen -- same as the rest of F125). Verified against a real running dev server with real earned points (screenshot walkthrough of both the pre-opt-in private state and the post-opt-in ranked state). Also fixed two test-fixture bugs surfaced while verifying under the full suite: this slices own integration tests were fixturing MATH-SEED chapter 1 (already flagged as shared/contested by F012s own migration note) instead of a dedicated isolated chapter, occasionally starving other tests (F118) of their own fixture question; and this sessions ad-hoc screenshot-verification scripts had left real leftover fixture rows in real Mathematics chapter 1 content, found and removed. Full suite 509/509 green. Not yet built: reward animation/sound, a parent-facing leaderboard view. [UPDATE 3] Reward animation/sound shipped: POST /api/attempts/:id/submit now returns points_earned ({points, coins}) whenever the just-confirmed evaluation actually paid out (the all-MCQ adaptive-paper auto-confirm path only -- null otherwise, since nothing has been confirmed yet for a parent-gated paper). /attempt/:id shows a coin badge on the results card (prefers-reduced-motion respected) and plays a short synthesized Web Audio chime (src/lib/reward-sound.ts -- no external audio asset, best-effort, never blocks showing the result). Covered by a new assertion in the existing adaptive-learning.integration.test.ts (the exact points/coins total for a controlled right/wrong mix), full suite still 509/509, and confirmed live against the real e2e adaptive-flow spec in isolation (that spec and happy-path both hit pre-existing, unrelated flakes on /profile-setup and under DB-pool contention when run concurrently with the full suite -- neither touches this change). Status stays In Progress: the one item left is a parent-facing leaderboard view. [UPDATE 4] User decision 2026-09-22: no parent-facing leaderboard view needed -- GET /api/leaderboard stays student-self only, by design, not a gap. Every stated AC item is built and verified (points by difficulty on MCQ submit, coin+sound reward, opt-in anonymous same-board/class/subject leaderboard, T09 kept intact). Status -&gt; Done.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(F127): usability pass -- navigation, student home, parent dashboard, loading states
- Shell: signed-in name + Sign out on every page; bottom tab bar below lg.
- /student: greeting header, Recommended next first, stat tiles, subjects
  collapsed until opened; no longer crashes on an error from /api/papers.
- /my-paper: Generate Assessment moved to a sticky bar below the chapters.
- /home: parent's pending actions first, recap as three numbers, next action
  per subject first with charts folded away, habit legend. Delivery Gap is
  now shown in marks (it was printed with a wrong "%" suffix).
- Skeleton placeholders replace the bare "Loading..." line on every screen.
- Tab 03: F127 added and marked Done; CLAUDE.md feature count updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ExamPrep_AI_Module_Development_Plan.xlsx
+++ b/docs/ExamPrep_AI_Module_Development_Plan.xlsx
@@ -10632,7 +10632,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K129"/>
+  <dimension ref="A1:K130"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
   <cols>
     <col width="10" customWidth="1" style="38" min="1" max="2"/>
@@ -17518,6 +17518,61 @@
       <c r="K129" t="inlineStr">
         <is>
           <t>Added 2026-09-23 at the owner's request. Lazy generation only -- an ~8,000 question MCQ bank is explained on demand, never bulk-backfilled. Cache lives in question_explanations (migration 0070).</t>
+        </is>
+      </c>
+    </row>
+    <row r="130" ht="15" customHeight="1" s="38">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>M14</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>F127</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Usability pass: navigation, student home, parent dashboard, loading states</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>As a parent or student I want every screen to show what to do next first, and to move between sections easily on a phone, so that the app is simple to use without explanation.</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>Sign out and the signed-in name are reachable from the shell on every page; below the lg breakpoint a bottom tab bar shows the main sections. Student home leads with Recommended next and papers to attempt, then four stat tiles, then needs-improvement/revise/strong, with subjects collapsed until opened. On /my-paper the Generate Assessment button stays in view in a sticky bar below the chapter list. Parent dashboard leads with what waits on the parent (Needs evaluation, Today's action), shows the recap as three numbers, puts each subject's next action first and folds its charts away, shows Delivery Gap in marks with a plain-language definition, and gives the habit dots a legend. Every screen shows skeleton placeholders instead of a bare "Loading..." line. No API, schema or permission changes.</t>
+        </is>
+      </c>
+      <c r="F130" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G130" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H130" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>S22</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K130" t="inlineStr">
+        <is>
+          <t>Added 2026-09-30 at the owner's request ("make it userfriendly"), after a UX review; the owner chose an in-place overhaul over a rewrite, student screens first. Also fixes a real display bug: /home printed delivery_gap (knowledge_score - actual_score, a count of marks) with a "%" suffix. /student no longer crashes when GET /api/papers returns an error body. e2e/adaptive-flow.spec.ts now opens the fixture subject before checking its concept, since subjects start collapsed. Full e2e (10) and unit (231) suites green.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: realign F126 row in tab 03, update feature count to 127, extend Status dropdown
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ExamPrep_AI_Module_Development_Plan.xlsx
+++ b/docs/ExamPrep_AI_Module_Development_Plan.xlsx
@@ -10649,7 +10649,7 @@
     <row r="1" ht="24" customHeight="1" s="38">
       <c r="A1" s="42" t="inlineStr">
         <is>
-          <t>03  Feature Backlog  —  124 features. Type Not Started / In Progress / Blocked / Done in column J.</t>
+          <t>03  Feature Backlog  —  127 features. Type Not Started / In Progress / Blocked / Done in column J.</t>
         </is>
       </c>
     </row>
@@ -17482,16 +17482,11 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Student</t>
+          <t>As a student reviewing my marked paper, I want to see why the correct answer is correct, so I learn the method instead of only learning that I was wrong.</t>
         </is>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>As a student reviewing my marked paper, I want to see why the correct answer is correct, so I learn the method instead of only learning that I was wrong.</t>
-        </is>
-      </c>
-      <c r="F129" t="inlineStr">
-        <is>
           <t>Given a paper whose marks are confirmed, when she opens a question on her result screen and asks for an explanation, then a short worked explanation is shown and cached per question and reused for every student who sees that question afterwards; questions that already carry a question_step_marks scheme use it verbatim with no AI call; with no AI provider configured nothing is invented and she is told it is unavailable; never available before marks are confirmed (T09 amendment 2026-09-22).</t>
         </is>
       </c>
@@ -17500,14 +17495,10 @@
           <t>M</t>
         </is>
       </c>
-      <c r="H129" s="10" t="inlineStr">
-        <is>
-          <t>AI-13</t>
-        </is>
-      </c>
+      <c r="H129" s="10" t="n"/>
       <c r="I129" t="inlineStr">
         <is>
-          <t>F049, F067</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="J129" t="inlineStr">
@@ -17517,7 +17508,7 @@
       </c>
       <c r="K129" t="inlineStr">
         <is>
-          <t>Added 2026-09-23 at the owner's request. Lazy generation only -- an ~8,000 question MCQ bank is explained on demand, never bulk-backfilled. Cache lives in question_explanations (migration 0070).</t>
+          <t>Added 2026-09-23 at the owner's request. Lazy generation only -- an ~8,000 question MCQ bank is explained on demand, never bulk-backfilled. Cache lives in question_explanations (migration 0070). AI layer: AI-13 (tab 07). Depends on F049, F067. (Row realigned 2026-09-30: values had been entered one column to the right, with a "Student" persona in the User Story column; priority and estimate were never recorded.)</t>
         </is>
       </c>
     </row>
@@ -17582,7 +17573,7 @@
     <mergeCell ref="A1:K1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="J4:J125" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J4:J130" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not Started,In Progress,Blocked,Done"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
feat(F128): Aurora visual theme -- 3D glass UI, gradient colours, interface sounds
- Original violet/pink/orange gradient palette with cyan and lime highlights,
  light and dark; drifting colour field behind every screen.
- Glass cards with layered shadows; chunky 3D buttons that press down;
  glowing gradient nav pill; gradient Recommended-next hero; colour-coded
  stat tiles; Outfit display font.
- Synthesized Web Audio tap/nav/select sounds on every button and link,
  with a remembered sound switch (also silences the F125 coin chime).
- Reduced-motion respected; printouts stay plain.
- Tab 03: F128 added and marked Done; CLAUDE.md feature count updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ExamPrep_AI_Module_Development_Plan.xlsx
+++ b/docs/ExamPrep_AI_Module_Development_Plan.xlsx
@@ -10632,7 +10632,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K130"/>
+  <dimension ref="A1:K131"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
   <cols>
     <col width="10" customWidth="1" style="38" min="1" max="2"/>
@@ -10649,7 +10649,7 @@
     <row r="1" ht="24" customHeight="1" s="38">
       <c r="A1" s="42" t="inlineStr">
         <is>
-          <t>03  Feature Backlog  —  127 features. Type Not Started / In Progress / Blocked / Done in column J.</t>
+          <t>03  Feature Backlog  —  128 features. Type Not Started / In Progress / Blocked / Done in column J.</t>
         </is>
       </c>
     </row>
@@ -17564,6 +17564,61 @@
       <c r="K130" t="inlineStr">
         <is>
           <t>Added 2026-09-30 at the owner's request ("make it userfriendly"), after a UX review; the owner chose an in-place overhaul over a rewrite, student screens first. Also fixes a real display bug: /home printed delivery_gap (knowledge_score - actual_score, a count of marks) with a "%" suffix. /student no longer crashes when GET /api/papers returns an error body. e2e/adaptive-flow.spec.ts now opens the fixture subject before checking its concept, since subjects start collapsed. Full e2e (10) and unit (231) suites green.</t>
+        </is>
+      </c>
+    </row>
+    <row r="131" ht="15" customHeight="1" s="38">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>M14</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>F128</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Aurora visual theme: 3D glass UI, gradient colours, interface sounds</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>As a student I want the app to look and sound exciting and modern, so that I enjoy opening it and practising every day.</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>Theme tokens (src/styles.css) define an original violet-pink-orange gradient palette with cyan and lime highlights, in light and dark mode; a slowly drifting colour field sits behind every screen; cards are translucent glass with layered shadows; primary buttons are chunky 3D buttons that press down on click; the active nav item is a glowing gradient pill; Recommended next is a gradient hero card; stat tiles are colour-coded. Every button, link and choice plays a short synthesized sound (Web Audio, no audio files); a sound switch next to the theme toggle turns sounds off, remembered per device, and also silences the F125 coin chime. Animations stop for anyone whose device asks for reduced motion. Printouts stay plain black-on-white. No franchise palette, character or typeface is imitated.</t>
+        </is>
+      </c>
+      <c r="F131" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G131" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H131" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>S22</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K131" t="inlineStr">
+        <is>
+          <t>Added 2026-09-30 at the owner's request ("most stunning, 3D layers... sound and colour effects" for students born after 2010). Headings now use Outfit instead of Fraunces. Checked with real screenshots (desktop, phone, dark mode). Full e2e (10) and unit (231) suites green.</t>
         </is>
       </c>
     </row>
@@ -17573,7 +17628,7 @@
     <mergeCell ref="A1:K1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="J4:J130" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J4:J131" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not Started,In Progress,Blocked,Done"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
feat(F128): calm pastel theme (beige, white, light pink, blue, yellow)
Replaces the bright Aurora palette at the owner's request: warm beige-white
base with soft pastel washes, one deep blue for actions, solid ink
headings, pastel stat tiles and badges. Heading font Plus Jakarta Sans.
Tab 03: F128 revised, F129 and F130 added; CLAUDE.md count updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ExamPrep_AI_Module_Development_Plan.xlsx
+++ b/docs/ExamPrep_AI_Module_Development_Plan.xlsx
@@ -10632,7 +10632,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K131"/>
+  <dimension ref="A1:K133"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
   <cols>
     <col width="10" customWidth="1" style="38" min="1" max="2"/>
@@ -10649,7 +10649,7 @@
     <row r="1" ht="24" customHeight="1" s="38">
       <c r="A1" s="42" t="inlineStr">
         <is>
-          <t>03  Feature Backlog  —  128 features. Type Not Started / In Progress / Blocked / Done in column J.</t>
+          <t>03  Feature Backlog  —  130 features. Type Not Started / In Progress / Blocked / Done in column J.</t>
         </is>
       </c>
     </row>
@@ -17580,17 +17580,17 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Aurora visual theme: 3D glass UI, gradient colours, interface sounds</t>
+          <t>Calm pastel visual theme: glass cards, 3D buttons, interface sounds</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>As a student I want the app to look and sound exciting and modern, so that I enjoy opening it and practising every day.</t>
+          <t>As a student I want the app to look calm, modern and pleasant, and to respond with gentle sounds, so that I enjoy opening it and practising every day.</t>
         </is>
       </c>
       <c r="E131" t="inlineStr">
         <is>
-          <t>Theme tokens (src/styles.css) define an original violet-pink-orange gradient palette with cyan and lime highlights, in light and dark mode; a slowly drifting colour field sits behind every screen; cards are translucent glass with layered shadows; primary buttons are chunky 3D buttons that press down on click; the active nav item is a glowing gradient pill; Recommended next is a gradient hero card; stat tiles are colour-coded. Every button, link and choice plays a short synthesized sound (Web Audio, no audio files); a sound switch next to the theme toggle turns sounds off, remembered per device, and also silences the F125 coin chime. Animations stop for anyone whose device asks for reduced motion. Printouts stay plain black-on-white. No franchise palette, character or typeface is imitated.</t>
+          <t>Theme tokens (src/styles.css) define an original calm palette -- warm beige/white base with soft light-pink, baby-blue and butter-yellow washes drifting slowly behind every screen -- and one deep blue for every action so buttons and links stay readable; light and dark mode. Cards are translucent glass with gentle shadows; primary buttons are 3D buttons that press down on click; the active nav item is a soft blue pill; stat tiles carry pastel accents. Every button, link and choice plays a short synthesized sound (Web Audio, no audio files); a sound switch next to the theme toggle turns sounds off, remembered per device, and also silences the F125 coin chime. Animations stop under reduced-motion. Printouts stay plain. No franchise palette, character or typeface is imitated.</t>
         </is>
       </c>
       <c r="F131" t="inlineStr">
@@ -17618,7 +17618,117 @@
       </c>
       <c r="K131" t="inlineStr">
         <is>
-          <t>Added 2026-09-30 at the owner's request ("most stunning, 3D layers... sound and colour effects" for students born after 2010). Headings now use Outfit instead of Fraunces. Checked with real screenshots (desktop, phone, dark mode). Full e2e (10) and unit (231) suites green.</t>
+          <t>Added 2026-09-30 at the owner's request. First shipped as a bright violet/pink/orange "Aurora" theme; revised the same day, at the owner's request, to calm pastels (beige, white, light pink, blue, yellow). Checked with real screenshots in light and dark mode.</t>
+        </is>
+      </c>
+    </row>
+    <row r="132" ht="15" customHeight="1" s="38">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>M09</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>F129</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Readable question typography, spelling-tolerant marking, "Report a problem"</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>As a student I want questions, answers and headings to look clearly different, not to lose marks for a spelling slip, and to be able to tell someone when a question or its marking is wrong, so that my marks reflect what I actually know.</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>Typography: headings in Plus Jakarta Sans, question text in Lexend a size above body text with a "Q1" badge, options as tappable tiles, answers in Manrope under small uppercase labels (YOUR ANSWER / CORRECT ANSWER) in tinted boxes -- on the answering, result and review screens. Spelling: a fill-in-the-blank answer that is the right word with a small slip (edits scale with length, first letter must match, numbers must match exactly) earns full marks; the AI grading and re-review prompts explicitly treat recognisable misspellings as correct. Report a problem: on every question, during the attempt and on the result, a student picks a reason (marked wrong but right / question has a mistake / answer key has a mistake / unclear / other) and writes 3-300 characters; one report per question per attempt; own attempt only. Reports never change a mark. Admins see their own household's reports (question, key and the student's answer side by side) at /admin/reports and mark them resolved/dismissed.</t>
+        </is>
+      </c>
+      <c r="F132" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G132" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H132" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>S22</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K132" t="inlineStr">
+        <is>
+          <t>Added 2026-09-30 at the owner's request. Root cause of the spelling complaint: fill_blank was marked by exact text match (scoring.ts), so "photosynthsis" scored 0. New table question_reports (migration 0071). Admin queue is household-scoped because admin is a household role here, not a cross-tenant superadmin (F083). Tests: question-reports.integration.test.ts, scoring.test.ts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="133" ht="15" customHeight="1" s="38">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>M07</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>F130</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>Student downloads her own question paper as PDF</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>As a student I want to download my question paper as a PDF so that I can print it or practise on paper.</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>A "Download this paper as PDF" button sits above the question paper on the attempt screen and on the result screen. GET /api/papers/:id/pdf now also accepts the student role, but only for a paper generated for her (a sibling's paper is 404) and never with the answer key (include_key from a student is 403). ?download=1 saves it under a readable file name.</t>
+        </is>
+      </c>
+      <c r="F133" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G133" s="9" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="H133" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>S22</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="K133" t="inlineStr">
+        <is>
+          <t>Added 2026-09-30 at the owner's request. The PDF template never receives answers or which option is correct, so the plain paper is within the T09 rule. Tests in papers-pdf.integration.test.ts.</t>
         </is>
       </c>
     </row>
@@ -17628,7 +17738,7 @@
     <mergeCell ref="A1:K1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="J4:J131" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J4:J133" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not Started,In Progress,Blocked,Done"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
feat(F131): Android app as a Trusted Web Activity
The Android app wraps the production web app in a Trusted Web Activity (TWA), so every web
feature ships in it on day one and web deploys reach it without a Play update. The owner
approved this approach on 2026-09-30.

- android/: TWA shell built on android-browser-helper, no Kotlin code. Includes splash,
  adaptive icons, notification delegation and a WebView fallback. appId and hostName live in
  gradle.properties and must be finalised before the first Play upload.
- /.well-known/assetlinks.json is served from ANDROID_PACKAGE_NAME + ANDROID_CERT_SHA256.
  It returns 404 until both are configured.
- public/sw.js + offline.html give an offline fallback page. The service worker never caches
  API data or answers.
- CI builds a debug APK on every run, plus a signed AAB/APK once the signing secrets are set.
- Tab 03 gains F131, and tab 01 revises "Native mobile apps: out of scope".

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ExamPrep_AI_Module_Development_Plan.xlsx
+++ b/docs/ExamPrep_AI_Module_Development_Plan.xlsx
@@ -9009,12 +9009,12 @@
       </c>
       <c r="C17" s="51" t="inlineStr">
         <is>
-          <t>Responsive web only. PWA install is acceptable; App Store submission is not in v1.</t>
+          <t>Responsive web only in v1. Revised 2026-09-30 at the owner's request: an Android app ships on Google Play as a Trusted Web Activity over the same web app (F131). iOS/App Store is still excluded.</t>
         </is>
       </c>
       <c r="D17" s="51" t="inlineStr">
         <is>
-          <t>Excluded</t>
+          <t>Revised (F131)</t>
         </is>
       </c>
     </row>
@@ -10632,7 +10632,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K133"/>
+  <dimension ref="A1:K134"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6328125" defaultRowHeight="14.5"/>
   <cols>
     <col width="10" customWidth="1" style="38" min="1" max="2"/>
@@ -10649,7 +10649,7 @@
     <row r="1" ht="24" customHeight="1" s="38">
       <c r="A1" s="42" t="inlineStr">
         <is>
-          <t>03  Feature Backlog  —  130 features. Type Not Started / In Progress / Blocked / Done in column J.</t>
+          <t>03  Feature Backlog  —  131 features. Type Not Started / In Progress / Blocked / Done in column J.</t>
         </is>
       </c>
     </row>
@@ -17729,6 +17729,61 @@
       <c r="K133" t="inlineStr">
         <is>
           <t>Added 2026-09-30 at the owner's request. The PDF template never receives answers or which option is correct, so the plain paper is within the T09 rule. Tests in papers-pdf.integration.test.ts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="134" ht="15" customHeight="1" s="38">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>M01</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>F131</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Android app on Google Play (Trusted Web Activity)</t>
+        </is>
+      </c>
+      <c r="D134" t="inlineStr">
+        <is>
+          <t>As a parent I want to install ExamPrep AI from the Google Play Store so that my child and I can open it like any other app on our Android phones.</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>An Android app, built as a Trusted Web Activity over the production web app, is published on Google Play. It opens full-screen with no browser URL bar, which proves Digital Asset Links is verified: /.well-known/assetlinks.json is served by the web app, and its SHA-256 fingerprints come from configuration, not code. Every web feature works inside it: sign-in (email and Google), taking an attempt, photographing a handwritten answer with the camera, and downloading a paper PDF. A service worker shows a friendly offline page when there is no network, and never caches API responses or answer data. Phones without a TWA-capable browser fall back to a WebView. A signed AAB is built in CI, never on a developer laptop, and the signing keystore is not in the repo. The Families Policy declarations, a public privacy policy URL and the Data Safety form are complete. iOS/App Store is still excluded.</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G134" s="9" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="H134" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>S23</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="K134" t="inlineStr">
+        <is>
+          <t>Added 2026-09-30 at the owner's request, reversing tab 01's 'Native mobile apps: out of scope v1'. TWA, not a native rewrite (owner approved): every web feature ships on day one and web deploys reach the app without a Play update. Owner arranging: personal Play Console account (needs a 12-tester, 14-day closed test before production) and a custom domain (the app is bound to its domain, so this must be set before the first Play upload).</t>
         </is>
       </c>
     </row>
@@ -17738,7 +17793,7 @@
     <mergeCell ref="A1:K1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="J4:J133" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J4:J134" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Not Started,In Progress,Blocked,Done"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>